<commit_message>
Add Period methods and tests
</commit_message>
<xml_diff>
--- a/tests/workbooks/test_date.xlsx
+++ b/tests/workbooks/test_date.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8258C8E4-7147-4C8B-B865-77B201E38E5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A3A3692-1E1E-42E5-AC8A-8386A5DFDB12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12135" yWindow="-14625" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4530" yWindow="-18405" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="qlPeriod" sheetId="1" r:id="rId1"/>
@@ -58,6 +58,17 @@
     </bk>
   </cellMetadata>
 </metadata>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t>37d</t>
+  </si>
+  <si>
+    <t>12M</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -373,19 +384,62 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="str" cm="1">
-        <f t="array" ref="A1">_xll.qlPeriod(3,"Months")</f>
-        <v>3M</v>
+      <c r="A1" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2">_xll.qlPeriod(37,"daYs")</f>
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" cm="1">
+        <f t="array" ref="A3">_xll.qlPeriodLength(A1)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="str" cm="1">
+        <f t="array" ref="A4">_xll.qlPeriodFrequency(A1)</f>
+        <v>ANNUAL</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="str" cm="1">
+        <f t="array" ref="A5">_xll.qlPeriodFrequency(A2)</f>
+        <v>OTHERFREQUENCY</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="str" cm="1">
+        <f t="array" ref="A6">_xll.qlPeriodNormalized(A1)</f>
+        <v>1Y</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="str" cm="1">
+        <f t="array" ref="A7">_xll.qlPeriodNormalized(A2)</f>
         <v>37D</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="str" cm="1">
+        <f t="array" ref="A8">_xll.qlPeriodUnits(A1)</f>
+        <v>MONTHS</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="str" cm="1">
+        <f t="array" ref="A9">_xll.qlPeriodUnits(A2)</f>
+        <v>DAYS</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Date and Date methods and tests
</commit_message>
<xml_diff>
--- a/tests/workbooks/test_date.xlsx
+++ b/tests/workbooks/test_date.xlsx
@@ -8,12 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A3A3692-1E1E-42E5-AC8A-8386A5DFDB12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AFEF087-6DAE-4D61-988B-982D70611DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4530" yWindow="-18405" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10425" yWindow="-19335" windowWidth="23040" windowHeight="16005" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="qlPeriod" sheetId="1" r:id="rId1"/>
+    <sheet name="qlDate" sheetId="2" r:id="rId2"/>
+    <sheet name="qlDateParser" sheetId="3" r:id="rId3"/>
+    <sheet name="qlPeriodParser" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -61,18 +64,120 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>37d</t>
   </si>
   <si>
     <t>12M</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Day</t>
+  </si>
+  <si>
+    <t>qlDate</t>
+  </si>
+  <si>
+    <t>qlDateWeekday</t>
+  </si>
+  <si>
+    <t>qlDateDayOfMonth</t>
+  </si>
+  <si>
+    <t>qlDateMonth</t>
+  </si>
+  <si>
+    <t>qlDateYear</t>
+  </si>
+  <si>
+    <t>qlDateDayOfYear</t>
+  </si>
+  <si>
+    <t>qlDateIsLeap</t>
+  </si>
+  <si>
+    <t>qlDateMinDate</t>
+  </si>
+  <si>
+    <t>qlDateMaxDate</t>
+  </si>
+  <si>
+    <t>qlDateTodaysDate</t>
+  </si>
+  <si>
+    <t>qlDateStartOfMonth</t>
+  </si>
+  <si>
+    <t>qlDateEndOfMonth</t>
+  </si>
+  <si>
+    <t>qlDateIsStartOfMonth</t>
+  </si>
+  <si>
+    <t>qlDateIsEndOfMonth</t>
+  </si>
+  <si>
+    <t>qlDateNextWeekday</t>
+  </si>
+  <si>
+    <t>Weekday</t>
+  </si>
+  <si>
+    <t>Tuesday</t>
+  </si>
+  <si>
+    <t>qlDateNthWeekday</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>String</t>
+  </si>
+  <si>
+    <t>ISO String</t>
+  </si>
+  <si>
+    <t>2024-04-12</t>
+  </si>
+  <si>
+    <t>qlDateParserParseFormatted</t>
+  </si>
+  <si>
+    <t>Format</t>
+  </si>
+  <si>
+    <t>12.04.2024</t>
+  </si>
+  <si>
+    <t>%d.%m.%Y</t>
+  </si>
+  <si>
+    <t>qlDateParserParseISO</t>
+  </si>
+  <si>
+    <t>Period String</t>
+  </si>
+  <si>
+    <t>qlPeriodParserParse</t>
+  </si>
+  <si>
+    <t>1y3M</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -102,8 +207,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -445,4 +553,285 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46906BE3-F11A-458F-9DD4-FCBD355E6523}">
+  <dimension ref="A1:B21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.33203125" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" cm="1">
+        <f t="array" ref="B4">_xll.qlDate(B1,B2,B3)</f>
+        <v>46159</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="str" cm="1">
+        <f t="array" ref="B5">_xll.qlDateWeekday(B4)</f>
+        <v>SUNDAY</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" cm="1">
+        <f t="array" ref="B6">_xll.qlDateDayOfMonth(B4)</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" cm="1">
+        <f t="array" ref="B7">_xll.qlDateDayOfYear(B4)</f>
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" cm="1">
+        <f t="array" ref="B8">_xll.qlDateMonth(B4)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" cm="1">
+        <f t="array" ref="B9">_xll.qlDateYear(B4)</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="b" cm="1">
+        <f t="array" ref="B10">_xll.qlDateIsLeap(B9-2)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="1" cm="1">
+        <f t="array" ref="B14">_xll.qlDateStartOfMonth(B4)</f>
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="1" cm="1">
+        <f t="array" ref="B15">_xll.qlDateEndOfMonth(B4)</f>
+        <v>46173</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="b" cm="1">
+        <f t="array" ref="B16">_xll.qlDateIsStartOfMonth(B14)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" t="b" cm="1">
+        <f t="array" ref="B17">_xll.qlDateIsEndOfMonth(B15)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="1" cm="1">
+        <f t="array" ref="B19">_xll.qlDateNextWeekday(B4,B18)</f>
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="1" cm="1">
+        <f t="array" ref="B21">_xll.qlDateNthWeekday(B20,B18,B8,B9)</f>
+        <v>46161</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F10FA8D3-46AE-49A1-A85A-03A63DBCD87C}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.77734375" customWidth="1"/>
+    <col min="2" max="2" width="19.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="3" cm="1">
+        <f t="array" ref="B4">_xll.qlDateParserParseFormatted(B1,B2)</f>
+        <v>45394</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="3" cm="1">
+        <f t="array" ref="B5">_xll.qlDateParserParseISO(B3)</f>
+        <v>45394</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD34B23F-20C4-4C32-94BC-89E68DE44435}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="str" cm="1">
+        <f t="array" ref="B2">_xll.qlPeriodParserParse(B1)</f>
+        <v>15M</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>